<commit_message>
feat(catalogo): disponibilidade em estoque / sob encomenda com prazo, na planilha de importação e na página do produto
Padrão in_stock (nada muda). Regra de compra (estoque) intacta. Migração aditiva.
</commit_message>
<xml_diff>
--- a/apps/web/public/modelos/modelo-importacao-produtos.xlsx
+++ b/apps/web/public/modelos/modelo-importacao-produtos.xlsx
@@ -77,6 +77,8 @@
     <col min="11" max="11" width="11" customWidth="1"/>
     <col min="12" max="12" width="15" customWidth="1"/>
     <col min="13" max="13" width="50" customWidth="1"/>
+    <col min="14" max="14" width="16" customWidth="1"/>
+    <col min="15" max="15" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -145,6 +147,16 @@
           <t xml:space="preserve">fotos</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">disponibilidade</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prazo_dias</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -198,6 +210,11 @@
           <t xml:space="preserve">geladeira-frente.jpg|geladeira-aberta.jpg</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">em_estoque</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -247,6 +264,14 @@
         <is>
           <t xml:space="preserve">https://exemplo-do-fornecedor.com.br/fotos/smartphone-preto.jpg</t>
         </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sob_encomenda</t>
+        </is>
+      </c>
+      <c r="O3">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -571,59 +596,75 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">disponibilidade</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">“em_estoque” (padrão) ou “sob_encomenda” (você compra do fornecedor depois da venda). Vazio = não muda. Não altera a regra de compra: continua valendo o estoque.</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sob_encomenda</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dicas</t>
-        </is>
-      </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
+          <t xml:space="preserve">prazo_dias</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Só se sob_encomenda</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dias úteis a mais até o envio quando sob encomenda (1 a 120). Aparece na página do produto.</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
+      <c r="A17" s="3"/>
       <c r="B17" s="3"/>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Apague as linhas EXEMPLO-001 e EXEMPLO-002 da aba Produtos (se esquecer, o sistema recusa essas linhas).</t>
-        </is>
-      </c>
+      <c r="C17" s="3"/>
       <c r="D17" s="3"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">Dicas</t>
         </is>
       </c>
       <c r="B18" s="3"/>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Não mude os nomes das colunas da primeira linha. Colunas fora desta lista são ignoradas.</t>
-        </is>
-      </c>
+      <c r="C18" s="3"/>
       <c r="D18" s="3"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Célula vazia não apaga o que já está salvo. Para corrigir só o preço de um produto, basta preencher sku e preco.</t>
+          <t xml:space="preserve">Apague as linhas EXEMPLO-001 e EXEMPLO-002 da aba Produtos (se esquecer, o sistema recusa essas linhas).</t>
         </is>
       </c>
       <c r="D19" s="3"/>
@@ -631,13 +672,13 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Máximo de 500 produtos por planilha. Se tiver mais, divida em arquivos.</t>
+          <t xml:space="preserve">Não mude os nomes das colunas da primeira linha. Colunas fora desta lista são ignoradas.</t>
         </is>
       </c>
       <c r="D20" s="3"/>
@@ -645,16 +686,44 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Célula vazia não apaga o que já está salvo. Para corrigir só o preço de um produto, basta preencher sku e preco.</t>
+        </is>
+      </c>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Máximo de 500 produtos por planilha. Se tiver mais, divida em arquivos.</t>
+        </is>
+      </c>
+      <c r="D22" s="3"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">A importação nunca apaga produtos nem fotos.</t>
         </is>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D23" s="3"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>